<commit_message>
Limit every results workbook to 5 sheets with the most informative content
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MCd92X1TQnJhwpdce7yB5m
</commit_message>
<xml_diff>
--- a/results/part1_step2_etl_pipeline/etl_results.xlsx
+++ b/results/part1_step2_etl_pipeline/etl_results.xlsx
@@ -9,12 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flags" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory_Timing" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception_Tests" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Dictionary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory_Timing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tests" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Dictionary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1137,197 +1134,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>rows_flagged</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pct_of_fact</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>meaning</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>flag_sales_imputed</t>
+          <t>Rows with stock known (weeks 2..260)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sales_Units was missing and recovered as Revenue / Price</t>
-        </is>
+        <v>7770</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>flag_zero_sales</t>
+          <t>Same-row view: sales &gt; inventory_level</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1329</v>
-      </c>
-      <c r="C3" t="n">
-        <v>17.04</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sales_Units = 0 (always a stock-out week: previous-row inventory = 0)</t>
-        </is>
+        <v>1929</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>flag_sales_pileup</t>
+          <t>Offset view: sales &gt; previous-row inventory</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2116</v>
-      </c>
-      <c r="C4" t="n">
-        <v>27.13</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sales_Units exactly 1,500 or 2,500 (pile-up caused by stock limits)</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>flag_inventory_pileup</t>
+          <t>Same-row view: inventory = 0 but sales &gt; 0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4143</v>
-      </c>
-      <c r="C5" t="n">
-        <v>53.12</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Inventory exactly 0 / 1,500 / 2,500 (clipped stock levels)</t>
-        </is>
+        <v>907</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>flag_stockout_week</t>
+          <t>Offset view: stock available = 0 weeks</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>1329</v>
       </c>
-      <c r="C6" t="n">
-        <v>17.04</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Stock available for the week (previous row's inventory) = 0 -&gt; sales forced to 0</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>flag_stock_limited</t>
+          <t xml:space="preserve">  ...of which sales = 0</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2813</v>
-      </c>
-      <c r="C7" t="n">
-        <v>36.06</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Sales &gt;= stock available (&gt; 0): demand is censored, true demand &gt;= sales</t>
-        </is>
+        <v>1329</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>flag_stock_unknown</t>
+          <t>Stock-limited weeks (sales &gt;= stock &gt; 0)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>First week of a product: stock available unknown</t>
-        </is>
+        <v>2813</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>flag_sales_outlier</t>
+          <t>Unconstrained weeks (sales &lt; stock)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>|robust z| &gt; 4 vs the product's own median (winsorised copy in sales_units_winsorized)</t>
-        </is>
+        <v>3628</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>flag_forecast_missing</t>
+          <t>Share of all known weeks that are censored</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>606</v>
-      </c>
-      <c r="C10" t="n">
-        <v>7.77</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Legacy Demand_Forecast missing (kept NULL)</t>
-        </is>
+        <v>0.533</v>
       </c>
     </row>
   </sheetData>
@@ -1341,113 +1254,744 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>group</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>expected</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>actual</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rows with stock known (weeks 2..260)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>7770</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>fact rows = products x weeks</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7800</v>
+      </c>
+      <c r="E2" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Same-row view: sales &gt; inventory_level</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1929</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dim_product rows</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Offset view: sales &gt; previous-row inventory</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dim_date rows</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>260</v>
+      </c>
+      <c r="D4" t="n">
+        <v>260</v>
+      </c>
+      <c r="E4" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Same-row view: inventory = 0 but sales &gt; 0</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>907</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>reconciliation: staging = fact + duplicates + quarantined</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>7839</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7839</v>
+      </c>
+      <c r="E5" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Offset view: stock available = 0 weeks</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1329</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>staging rows = raw file rows</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7839</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7839</v>
+      </c>
+      <c r="E6" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ...of which sales = 0</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1329</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>foreign-key violations</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Stock-limited weeks (sales &gt;= stock &gt; 0)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2813</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>duplicate (product, week) keys</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Unconstrained weeks (sales &lt; stock)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>3628</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NULL sales_units</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Share of all known weeks that are censored</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.533</v>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sales &gt; stock available (timing violations)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>stock-out weeks (stock = 0) where sales != 0</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>revenue != sales x price</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>gross_profit != revenue - sales x cogs</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>revenue_growth is inf / not finite</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>sum(revenue) DB vs pandas (abs diff)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>flag counts DB vs pandas (abs diff)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Database validation</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>dq log rows for quarantined = quarantine table rows</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>row 2: quarantined with 'non_positive_unit_price'</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>non_positive_unit_price</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>non_positive_unit_price</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>row 3: quarantined with 'missing_product'</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>missing_product</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>missing_product</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>row 4: quarantined with 'invalid_week'</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>invalid_week</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>invalid_week</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>row 5: quarantined with 'invalid_week'</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>invalid_week</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>invalid_week</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>row 6: quarantined with 'sales_unrecoverable'</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>sales_unrecoverable</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>sales_unrecoverable</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>row 7: quarantined with 'negative_sales_units'</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>negative_sales_units</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>negative_sales_units</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>row 11: quarantined with 'missing_inventory_level'</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>missing_inventory_level</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>missing_inventory_level</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>row 7840: quarantined with 'conflicting_duplicate_key'</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>conflicting_duplicate_key</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>conflicting_duplicate_key</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>row 1: corrupt 'abc' sales -&gt; recovered from revenue/price</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>recovered</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>recovered</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>row 10: corrupt forecast 'n/a' -&gt; NULL + logged</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>set_null</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>set_null</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>exact duplicate row dropped</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>bad rows never reach the fact table</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>missing input file -&gt; ExtractError</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ExtractError</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ExtractError</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>missing column -&gt; SchemaError</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SchemaError</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SchemaError</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Exception handling</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>unreadable file -&gt; ExtractError</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ExtractError</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ExtractError</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1456,638 +2000,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>expected</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>actual</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>row 2: quarantined with 'non_positive_unit_price'</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>non_positive_unit_price</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>non_positive_unit_price</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>row 3: quarantined with 'missing_product'</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>missing_product</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>missing_product</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>row 4: quarantined with 'invalid_week'</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>invalid_week</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>invalid_week</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>row 5: quarantined with 'invalid_week'</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>invalid_week</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>invalid_week</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>row 6: quarantined with 'sales_unrecoverable'</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>sales_unrecoverable</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>sales_unrecoverable</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>row 7: quarantined with 'negative_sales_units'</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>negative_sales_units</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>negative_sales_units</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>row 11: quarantined with 'missing_inventory_level'</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>missing_inventory_level</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>missing_inventory_level</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>row 7840: quarantined with 'conflicting_duplicate_key'</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>conflicting_duplicate_key</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>conflicting_duplicate_key</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>row 1: corrupt 'abc' sales -&gt; recovered from revenue/price</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>recovered</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>recovered</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>row 10: corrupt forecast 'n/a' -&gt; NULL + logged</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>set_null</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>set_null</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>exact duplicate row dropped</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>bad rows never reach the fact table</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>missing input file -&gt; ExtractError</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ExtractError</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>ExtractError</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>missing column -&gt; SchemaError</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SchemaError</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>SchemaError</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>unreadable file -&gt; ExtractError</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ExtractError</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>ExtractError</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="59" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>expected</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>actual</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>fact rows = products x weeks</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>7800</v>
-      </c>
-      <c r="C2" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D2" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>dim_product rows</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>30</v>
-      </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
-      <c r="D3" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>dim_date rows</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>260</v>
-      </c>
-      <c r="C4" t="n">
-        <v>260</v>
-      </c>
-      <c r="D4" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>reconciliation: staging = fact + duplicates + quarantined</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>7839</v>
-      </c>
-      <c r="C5" t="n">
-        <v>7839</v>
-      </c>
-      <c r="D5" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>staging rows = raw file rows</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>7839</v>
-      </c>
-      <c r="C6" t="n">
-        <v>7839</v>
-      </c>
-      <c r="D6" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>foreign-key violations</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>duplicate (product, week) keys</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>NULL sales_units</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>sales &gt; stock available (timing violations)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>stock-out weeks (stock = 0) where sales != 0</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>revenue != sales x price</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>gross_profit != revenue - sales x cogs</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>revenue_growth is inf / not finite</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>sum(revenue) DB vs pandas (abs diff)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>flag counts DB vs pandas (abs diff)</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>dq log rows for quarantined = quarantine table rows</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3866,261 +3778,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="130" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Topic</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Dates</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Source has only Week 1-260; a synthetic calendar is used (week 1 = Monday 2020-01-06). Calendar attributes (year, month, season) are therefore illustrative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Flag, don't delete</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Zero-sales, pile-up, inventory-inconsistent and outlier rows are kept and flagged so downstream models/pricing can decide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>A3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Duplicates</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>A row duplicated on (product, week) with identical values is a load duplicate; with different values it is ambiguous and quarantined.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>A4</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Sales recovery</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Revenue = Sales x Price holds for 100% of rows, so missing Sales_Units = ROUND(Revenue / Price).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Demand_Forecast</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Legacy baseline; missing values are NOT imputed (it is only a benchmark / feature).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>A6</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Derived KPIs</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Revenue, Gross_Profit, GPM, turnover and growth are recomputed; originals of turnover/growth kept as *_src.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>A7</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Inventory turnover</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Defined as units sold / stock available for those sales (= COGS sold / stock valued at unit COGS); source definition unknown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>A8</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Outliers</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Per-product robust z-score (median / MAD) &gt; 4; flagged and winsorised in a separate column only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>A9</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Pile-ups at 1,500 / 2,500</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sales capped by available stock (sales never exceed the previous row's inventory); demand in those weeks is right-censored.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>A10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Product categories</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Not in the source; mapped manually from product names (CATEGORY_MAP).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>A11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Operating profit</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Opex not provided; implied_opex = gross_profit - operating_profit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>A12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>SQLite, rebuilt from scratch on every run (idempotent); loaded in a single transaction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>A13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Inventory timing</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Inventory_Level in row t-1 is the stock available for week t's sales (sales never exceed it, stock = 0 always means sales = 0). Treated as a one-week offset in the source; original inventory_level is kept unchanged.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>